<commit_message>
Week 1 Saturday paper: balance the option lengths on nine items
The audit now asks that, past 30 characters, a Saturday item's shortest option reach 60
percent of its longest, and nine Week 1 items fell short. paper_edits.yaml proposes each fix
in the W1 block, with the lengths before and after: Q10, Q13, Q30, Q43 and Q44 give a short
distractor the belief behind it, Q49 shortens its long distractor and names the mean in the
short one, and Q15 and Q26 bring every option under 30 characters. On Q16 both ends were
keyed options, so keyed option a now names the weeks, with its meaning and its letter
unchanged. Stems and keys stay as the bank has them, and the key's notes answer the new
wording. The Word paper and key are rebuilt on the diagnostic format.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7zaoR4dQ5pzBFnsX549JQ
</commit_message>
<xml_diff>
--- a/content/W01/SAT/answer-key/C2_W01_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W01/SAT/answer-key/C2_W01_SAT_item_analysis_TRAINER.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discussion" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tags" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seats" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratings" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -69,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -81,6 +84,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9506,4 +9510,1508 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Step one: each part's rating beside its score</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Type each seat's ratings, 1 to 4, from the answer sheet; the rates on the right are computed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>5</v>
+      </c>
+      <c r="N3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 1</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 2</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 3</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 4</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 5</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 6</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 1</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 2</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 3</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 4</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 5</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="I5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$5:$BC$5))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$5:$BC$5=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$5:$BC$5)))</f>
+        <v/>
+      </c>
+      <c r="J5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$5:$BC$5))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$5:$BC$5=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$5:$BC$5)))</f>
+        <v/>
+      </c>
+      <c r="K5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$5:$BC$5))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$5:$BC$5=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$5:$BC$5)))</f>
+        <v/>
+      </c>
+      <c r="L5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$5:$BC$5))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$5:$BC$5=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$5:$BC$5)))</f>
+        <v/>
+      </c>
+      <c r="M5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$5:$BC$5))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$5:$BC$5=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$5:$BC$5)))</f>
+        <v/>
+      </c>
+      <c r="N5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$5:$BC$5))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$5:$BC$5=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$5:$BC$5)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="I6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$6:$BC$6))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$6:$BC$6=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$6:$BC$6)))</f>
+        <v/>
+      </c>
+      <c r="J6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$6:$BC$6))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$6:$BC$6=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$6:$BC$6)))</f>
+        <v/>
+      </c>
+      <c r="K6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$6:$BC$6))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$6:$BC$6=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$6:$BC$6)))</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$6:$BC$6))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$6:$BC$6=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$6:$BC$6)))</f>
+        <v/>
+      </c>
+      <c r="M6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$6:$BC$6))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$6:$BC$6=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$6:$BC$6)))</f>
+        <v/>
+      </c>
+      <c r="N6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$6:$BC$6))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$6:$BC$6=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$6:$BC$6)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="I7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$7:$BC$7))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$7:$BC$7=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$7:$BC$7)))</f>
+        <v/>
+      </c>
+      <c r="J7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$7:$BC$7))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$7:$BC$7=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$7:$BC$7)))</f>
+        <v/>
+      </c>
+      <c r="K7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$7:$BC$7))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$7:$BC$7=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$7:$BC$7)))</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$7:$BC$7))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$7:$BC$7=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$7:$BC$7)))</f>
+        <v/>
+      </c>
+      <c r="M7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$7:$BC$7))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$7:$BC$7=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$7:$BC$7)))</f>
+        <v/>
+      </c>
+      <c r="N7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$7:$BC$7))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$7:$BC$7=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$7:$BC$7)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="I8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$8:$BC$8))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$8:$BC$8=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$8:$BC$8)))</f>
+        <v/>
+      </c>
+      <c r="J8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$8:$BC$8))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$8:$BC$8=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$8:$BC$8)))</f>
+        <v/>
+      </c>
+      <c r="K8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$8:$BC$8))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$8:$BC$8=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$8:$BC$8)))</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$8:$BC$8))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$8:$BC$8=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$8:$BC$8)))</f>
+        <v/>
+      </c>
+      <c r="M8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$8:$BC$8))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$8:$BC$8=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$8:$BC$8)))</f>
+        <v/>
+      </c>
+      <c r="N8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$8:$BC$8))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$8:$BC$8=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$8:$BC$8)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="I9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$9:$BC$9))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$9:$BC$9=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$9:$BC$9)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$9:$BC$9))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$9:$BC$9=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$9:$BC$9)))</f>
+        <v/>
+      </c>
+      <c r="K9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$9:$BC$9))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$9:$BC$9=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$9:$BC$9)))</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$9:$BC$9))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$9:$BC$9=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$9:$BC$9)))</f>
+        <v/>
+      </c>
+      <c r="M9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$9:$BC$9))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$9:$BC$9=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$9:$BC$9)))</f>
+        <v/>
+      </c>
+      <c r="N9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$9:$BC$9))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$9:$BC$9=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$9:$BC$9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="I10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$10:$BC$10))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$10:$BC$10=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$10:$BC$10)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$10:$BC$10))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$10:$BC$10=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$10:$BC$10)))</f>
+        <v/>
+      </c>
+      <c r="K10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$10:$BC$10))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$10:$BC$10=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$10:$BC$10)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$10:$BC$10))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$10:$BC$10=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$10:$BC$10)))</f>
+        <v/>
+      </c>
+      <c r="M10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$10:$BC$10))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$10:$BC$10=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$10:$BC$10)))</f>
+        <v/>
+      </c>
+      <c r="N10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$10:$BC$10))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$10:$BC$10=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$10:$BC$10)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="I11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$11:$BC$11))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$11:$BC$11=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$11:$BC$11)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$11:$BC$11))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$11:$BC$11=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$11:$BC$11)))</f>
+        <v/>
+      </c>
+      <c r="K11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$11:$BC$11))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$11:$BC$11=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$11:$BC$11)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$11:$BC$11))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$11:$BC$11=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$11:$BC$11)))</f>
+        <v/>
+      </c>
+      <c r="M11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$11:$BC$11))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$11:$BC$11=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$11:$BC$11)))</f>
+        <v/>
+      </c>
+      <c r="N11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$11:$BC$11))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$11:$BC$11=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$11:$BC$11)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="I12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$12:$BC$12))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$12:$BC$12=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$12:$BC$12)))</f>
+        <v/>
+      </c>
+      <c r="J12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$12:$BC$12))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$12:$BC$12=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$12:$BC$12)))</f>
+        <v/>
+      </c>
+      <c r="K12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$12:$BC$12))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$12:$BC$12=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$12:$BC$12)))</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$12:$BC$12))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$12:$BC$12=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$12:$BC$12)))</f>
+        <v/>
+      </c>
+      <c r="M12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$12:$BC$12))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$12:$BC$12=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$12:$BC$12)))</f>
+        <v/>
+      </c>
+      <c r="N12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$12:$BC$12))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$12:$BC$12=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$12:$BC$12)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="I13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$13:$BC$13))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$13:$BC$13=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$13:$BC$13)))</f>
+        <v/>
+      </c>
+      <c r="J13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$13:$BC$13))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$13:$BC$13=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$13:$BC$13)))</f>
+        <v/>
+      </c>
+      <c r="K13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$13:$BC$13))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$13:$BC$13=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$13:$BC$13)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$13:$BC$13))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$13:$BC$13=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$13:$BC$13)))</f>
+        <v/>
+      </c>
+      <c r="M13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$13:$BC$13))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$13:$BC$13=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$13:$BC$13)))</f>
+        <v/>
+      </c>
+      <c r="N13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$13:$BC$13))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$13:$BC$13=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$13:$BC$13)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="I14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$14:$BC$14))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$14:$BC$14=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$14:$BC$14)))</f>
+        <v/>
+      </c>
+      <c r="J14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$14:$BC$14))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$14:$BC$14=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$14:$BC$14)))</f>
+        <v/>
+      </c>
+      <c r="K14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$14:$BC$14))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$14:$BC$14=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$14:$BC$14)))</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$14:$BC$14))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$14:$BC$14=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$14:$BC$14)))</f>
+        <v/>
+      </c>
+      <c r="M14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$14:$BC$14))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$14:$BC$14=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$14:$BC$14)))</f>
+        <v/>
+      </c>
+      <c r="N14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$14:$BC$14))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$14:$BC$14=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$14:$BC$14)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="I15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$15:$BC$15))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$15:$BC$15=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$15:$BC$15)))</f>
+        <v/>
+      </c>
+      <c r="J15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$15:$BC$15))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$15:$BC$15=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$15:$BC$15)))</f>
+        <v/>
+      </c>
+      <c r="K15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$15:$BC$15))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$15:$BC$15=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$15:$BC$15)))</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$15:$BC$15))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$15:$BC$15=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$15:$BC$15)))</f>
+        <v/>
+      </c>
+      <c r="M15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$15:$BC$15))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$15:$BC$15=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$15:$BC$15)))</f>
+        <v/>
+      </c>
+      <c r="N15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$15:$BC$15))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$15:$BC$15=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$15:$BC$15)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="I16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$16:$BC$16))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$16:$BC$16=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$16:$BC$16)))</f>
+        <v/>
+      </c>
+      <c r="J16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$16:$BC$16))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$16:$BC$16=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$16:$BC$16)))</f>
+        <v/>
+      </c>
+      <c r="K16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$16:$BC$16))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$16:$BC$16=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$16:$BC$16)))</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$16:$BC$16))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$16:$BC$16=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$16:$BC$16)))</f>
+        <v/>
+      </c>
+      <c r="M16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$16:$BC$16))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$16:$BC$16=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$16:$BC$16)))</f>
+        <v/>
+      </c>
+      <c r="N16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$16:$BC$16))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$16:$BC$16=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$16:$BC$16)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="I17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$17:$BC$17))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$17:$BC$17=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$17:$BC$17)))</f>
+        <v/>
+      </c>
+      <c r="J17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$17:$BC$17))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$17:$BC$17=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$17:$BC$17)))</f>
+        <v/>
+      </c>
+      <c r="K17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$17:$BC$17))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$17:$BC$17=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$17:$BC$17)))</f>
+        <v/>
+      </c>
+      <c r="L17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$17:$BC$17))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$17:$BC$17=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$17:$BC$17)))</f>
+        <v/>
+      </c>
+      <c r="M17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$17:$BC$17))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$17:$BC$17=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$17:$BC$17)))</f>
+        <v/>
+      </c>
+      <c r="N17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$17:$BC$17))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$17:$BC$17=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$17:$BC$17)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="I18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$18:$BC$18))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$18:$BC$18=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$18:$BC$18)))</f>
+        <v/>
+      </c>
+      <c r="J18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$18:$BC$18))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$18:$BC$18=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$18:$BC$18)))</f>
+        <v/>
+      </c>
+      <c r="K18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$18:$BC$18))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$18:$BC$18=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$18:$BC$18)))</f>
+        <v/>
+      </c>
+      <c r="L18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$18:$BC$18))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$18:$BC$18=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$18:$BC$18)))</f>
+        <v/>
+      </c>
+      <c r="M18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$18:$BC$18))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$18:$BC$18=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$18:$BC$18)))</f>
+        <v/>
+      </c>
+      <c r="N18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$18:$BC$18))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$18:$BC$18=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$18:$BC$18)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="I19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$19:$BC$19))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$19:$BC$19=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$19:$BC$19)))</f>
+        <v/>
+      </c>
+      <c r="J19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$19:$BC$19))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$19:$BC$19=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$19:$BC$19)))</f>
+        <v/>
+      </c>
+      <c r="K19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$19:$BC$19))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$19:$BC$19=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$19:$BC$19)))</f>
+        <v/>
+      </c>
+      <c r="L19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$19:$BC$19))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$19:$BC$19=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$19:$BC$19)))</f>
+        <v/>
+      </c>
+      <c r="M19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$19:$BC$19))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$19:$BC$19=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$19:$BC$19)))</f>
+        <v/>
+      </c>
+      <c r="N19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$19:$BC$19))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$19:$BC$19=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$19:$BC$19)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="I20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$20:$BC$20))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$20:$BC$20=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$20:$BC$20)))</f>
+        <v/>
+      </c>
+      <c r="J20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$20:$BC$20))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$20:$BC$20=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$20:$BC$20)))</f>
+        <v/>
+      </c>
+      <c r="K20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$20:$BC$20))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$20:$BC$20=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$20:$BC$20)))</f>
+        <v/>
+      </c>
+      <c r="L20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$20:$BC$20))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$20:$BC$20=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$20:$BC$20)))</f>
+        <v/>
+      </c>
+      <c r="M20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$20:$BC$20))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$20:$BC$20=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$20:$BC$20)))</f>
+        <v/>
+      </c>
+      <c r="N20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$20:$BC$20))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$20:$BC$20=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$20:$BC$20)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="I21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$21:$BC$21))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$21:$BC$21=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$21:$BC$21)))</f>
+        <v/>
+      </c>
+      <c r="J21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$21:$BC$21))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$21:$BC$21=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$21:$BC$21)))</f>
+        <v/>
+      </c>
+      <c r="K21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$21:$BC$21))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$21:$BC$21=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$21:$BC$21)))</f>
+        <v/>
+      </c>
+      <c r="L21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$21:$BC$21))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$21:$BC$21=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$21:$BC$21)))</f>
+        <v/>
+      </c>
+      <c r="M21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$21:$BC$21))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$21:$BC$21=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$21:$BC$21)))</f>
+        <v/>
+      </c>
+      <c r="N21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$21:$BC$21))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$21:$BC$21=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$21:$BC$21)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="I22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$22:$BC$22))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$22:$BC$22=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$22:$BC$22)))</f>
+        <v/>
+      </c>
+      <c r="J22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$22:$BC$22))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$22:$BC$22=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$22:$BC$22)))</f>
+        <v/>
+      </c>
+      <c r="K22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$22:$BC$22))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$22:$BC$22=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$22:$BC$22)))</f>
+        <v/>
+      </c>
+      <c r="L22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$22:$BC$22))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$22:$BC$22=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$22:$BC$22)))</f>
+        <v/>
+      </c>
+      <c r="M22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$22:$BC$22))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$22:$BC$22=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$22:$BC$22)))</f>
+        <v/>
+      </c>
+      <c r="N22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$22:$BC$22))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$22:$BC$22=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$22:$BC$22)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="I23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$23:$BC$23))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$23:$BC$23=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$23:$BC$23)))</f>
+        <v/>
+      </c>
+      <c r="J23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$23:$BC$23))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$23:$BC$23=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$23:$BC$23)))</f>
+        <v/>
+      </c>
+      <c r="K23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$23:$BC$23))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$23:$BC$23=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$23:$BC$23)))</f>
+        <v/>
+      </c>
+      <c r="L23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$23:$BC$23))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$23:$BC$23=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$23:$BC$23)))</f>
+        <v/>
+      </c>
+      <c r="M23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$23:$BC$23))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$23:$BC$23=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$23:$BC$23)))</f>
+        <v/>
+      </c>
+      <c r="N23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$23:$BC$23))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$23:$BC$23=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$23:$BC$23)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+      <c r="I24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$24:$BC$24))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$24:$BC$24=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$24:$BC$24)))</f>
+        <v/>
+      </c>
+      <c r="J24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$24:$BC$24))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$24:$BC$24=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$24:$BC$24)))</f>
+        <v/>
+      </c>
+      <c r="K24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$24:$BC$24))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$24:$BC$24=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$24:$BC$24)))</f>
+        <v/>
+      </c>
+      <c r="L24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$24:$BC$24))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$24:$BC$24=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$24:$BC$24)))</f>
+        <v/>
+      </c>
+      <c r="M24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$24:$BC$24))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$24:$BC$24=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$24:$BC$24)))</f>
+        <v/>
+      </c>
+      <c r="N24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$24:$BC$24))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$24:$BC$24=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$24:$BC$24)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="I25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$25:$BC$25))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$25:$BC$25=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$25:$BC$25)))</f>
+        <v/>
+      </c>
+      <c r="J25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$25:$BC$25))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$25:$BC$25=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$25:$BC$25)))</f>
+        <v/>
+      </c>
+      <c r="K25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$25:$BC$25))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$25:$BC$25=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$25:$BC$25)))</f>
+        <v/>
+      </c>
+      <c r="L25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$25:$BC$25))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$25:$BC$25=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$25:$BC$25)))</f>
+        <v/>
+      </c>
+      <c r="M25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$25:$BC$25))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$25:$BC$25=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$25:$BC$25)))</f>
+        <v/>
+      </c>
+      <c r="N25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$25:$BC$25))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$25:$BC$25=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$25:$BC$25)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="5" t="n"/>
+      <c r="I26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$26:$BC$26))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$26:$BC$26=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$26:$BC$26)))</f>
+        <v/>
+      </c>
+      <c r="J26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$26:$BC$26))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$26:$BC$26=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$26:$BC$26)))</f>
+        <v/>
+      </c>
+      <c r="K26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$26:$BC$26))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$26:$BC$26=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$26:$BC$26)))</f>
+        <v/>
+      </c>
+      <c r="L26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$26:$BC$26))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$26:$BC$26=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$26:$BC$26)))</f>
+        <v/>
+      </c>
+      <c r="M26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$26:$BC$26))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$26:$BC$26=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$26:$BC$26)))</f>
+        <v/>
+      </c>
+      <c r="N26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$26:$BC$26))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$26:$BC$26=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$26:$BC$26)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="I27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$27:$BC$27))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$27:$BC$27=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$27:$BC$27)))</f>
+        <v/>
+      </c>
+      <c r="J27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$27:$BC$27))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$27:$BC$27=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$27:$BC$27)))</f>
+        <v/>
+      </c>
+      <c r="K27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$27:$BC$27))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$27:$BC$27=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$27:$BC$27)))</f>
+        <v/>
+      </c>
+      <c r="L27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$27:$BC$27))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$27:$BC$27=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$27:$BC$27)))</f>
+        <v/>
+      </c>
+      <c r="M27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$27:$BC$27))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$27:$BC$27=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$27:$BC$27)))</f>
+        <v/>
+      </c>
+      <c r="N27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$27:$BC$27))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$27:$BC$27=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$27:$BC$27)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="I28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$28:$BC$28))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$28:$BC$28=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$28:$BC$28)))</f>
+        <v/>
+      </c>
+      <c r="J28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$28:$BC$28))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$28:$BC$28=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$28:$BC$28)))</f>
+        <v/>
+      </c>
+      <c r="K28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$28:$BC$28))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$28:$BC$28=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$28:$BC$28)))</f>
+        <v/>
+      </c>
+      <c r="L28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$28:$BC$28))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$28:$BC$28=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$28:$BC$28)))</f>
+        <v/>
+      </c>
+      <c r="M28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$28:$BC$28))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$28:$BC$28=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$28:$BC$28)))</f>
+        <v/>
+      </c>
+      <c r="N28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$28:$BC$28))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$28:$BC$28=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$28:$BC$28)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="I29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$29:$BC$29))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$29:$BC$29=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$29:$BC$29)))</f>
+        <v/>
+      </c>
+      <c r="J29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$29:$BC$29))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$29:$BC$29=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$29:$BC$29)))</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$29:$BC$29))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$29:$BC$29=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$29:$BC$29)))</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$29:$BC$29))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$29:$BC$29=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$29:$BC$29)))</f>
+        <v/>
+      </c>
+      <c r="M29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$29:$BC$29))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$29:$BC$29=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$29:$BC$29)))</f>
+        <v/>
+      </c>
+      <c r="N29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$29:$BC$29))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$29:$BC$29=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$29:$BC$29)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="I30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$30:$BC$30))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$30:$BC$30=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$30:$BC$30)))</f>
+        <v/>
+      </c>
+      <c r="J30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$30:$BC$30))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$30:$BC$30=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$30:$BC$30)))</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$30:$BC$30))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$30:$BC$30=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$30:$BC$30)))</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$30:$BC$30))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$30:$BC$30=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$30:$BC$30)))</f>
+        <v/>
+      </c>
+      <c r="M30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$30:$BC$30))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$30:$BC$30=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$30:$BC$30)))</f>
+        <v/>
+      </c>
+      <c r="N30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$30:$BC$30))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$30:$BC$30=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$30:$BC$30)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="I31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$31:$BC$31))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$31:$BC$31=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$31:$BC$31)))</f>
+        <v/>
+      </c>
+      <c r="J31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$31:$BC$31))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$31:$BC$31=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$31:$BC$31)))</f>
+        <v/>
+      </c>
+      <c r="K31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$31:$BC$31))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$31:$BC$31=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$31:$BC$31)))</f>
+        <v/>
+      </c>
+      <c r="L31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$31:$BC$31))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$31:$BC$31=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$31:$BC$31)))</f>
+        <v/>
+      </c>
+      <c r="M31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$31:$BC$31))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$31:$BC$31=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$31:$BC$31)))</f>
+        <v/>
+      </c>
+      <c r="N31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$31:$BC$31))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$31:$BC$31=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$31:$BC$31)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="I32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$32:$BC$32))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$32:$BC$32=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$32:$BC$32)))</f>
+        <v/>
+      </c>
+      <c r="J32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$32:$BC$32))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$32:$BC$32=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$32:$BC$32)))</f>
+        <v/>
+      </c>
+      <c r="K32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$32:$BC$32))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$32:$BC$32=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$32:$BC$32)))</f>
+        <v/>
+      </c>
+      <c r="L32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$32:$BC$32))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$32:$BC$32=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$32:$BC$32)))</f>
+        <v/>
+      </c>
+      <c r="M32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$32:$BC$32))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$32:$BC$32=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$32:$BC$32)))</f>
+        <v/>
+      </c>
+      <c r="N32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$32:$BC$32))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$32:$BC$32=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$32:$BC$32)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="I33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$33:$BC$33))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$33:$BC$33=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$33:$BC$33)))</f>
+        <v/>
+      </c>
+      <c r="J33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$33:$BC$33))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$33:$BC$33=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$33:$BC$33)))</f>
+        <v/>
+      </c>
+      <c r="K33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$33:$BC$33))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$33:$BC$33=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$33:$BC$33)))</f>
+        <v/>
+      </c>
+      <c r="L33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$33:$BC$33))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$33:$BC$33=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$33:$BC$33)))</f>
+        <v/>
+      </c>
+      <c r="M33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$33:$BC$33))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$33:$BC$33=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$33:$BC$33)))</f>
+        <v/>
+      </c>
+      <c r="N33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$33:$BC$33))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$33:$BC$33=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$33:$BC$33)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
+      <c r="I34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$34:$BC$34))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$34:$BC$34=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$34:$BC$34)))</f>
+        <v/>
+      </c>
+      <c r="J34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$34:$BC$34))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$34:$BC$34=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$34:$BC$34)))</f>
+        <v/>
+      </c>
+      <c r="K34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$34:$BC$34))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$34:$BC$34=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$34:$BC$34)))</f>
+        <v/>
+      </c>
+      <c r="L34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$34:$BC$34))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$34:$BC$34=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$34:$BC$34)))</f>
+        <v/>
+      </c>
+      <c r="M34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$34:$BC$34))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$34:$BC$34=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$34:$BC$34)))</f>
+        <v/>
+      </c>
+      <c r="N34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$34:$BC$34))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$34:$BC$34=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$34:$BC$34)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
+      <c r="I35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$35:$BC$35))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$35:$BC$35=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$35:$BC$35)))</f>
+        <v/>
+      </c>
+      <c r="J35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$35:$BC$35))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$35:$BC$35=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$35:$BC$35)))</f>
+        <v/>
+      </c>
+      <c r="K35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$35:$BC$35))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$35:$BC$35=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$35:$BC$35)))</f>
+        <v/>
+      </c>
+      <c r="L35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$35:$BC$35))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$35:$BC$35=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$35:$BC$35)))</f>
+        <v/>
+      </c>
+      <c r="M35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$35:$BC$35))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$35:$BC$35=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$35:$BC$35)))</f>
+        <v/>
+      </c>
+      <c r="N35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$35:$BC$35))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$35:$BC$35=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$35:$BC$35)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="I36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$36:$BC$36))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$36:$BC$36=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$36:$BC$36)))</f>
+        <v/>
+      </c>
+      <c r="J36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$36:$BC$36))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$36:$BC$36=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$36:$BC$36)))</f>
+        <v/>
+      </c>
+      <c r="K36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$36:$BC$36))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$36:$BC$36=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$36:$BC$36)))</f>
+        <v/>
+      </c>
+      <c r="L36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$36:$BC$36))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$36:$BC$36=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$36:$BC$36)))</f>
+        <v/>
+      </c>
+      <c r="M36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$36:$BC$36))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$36:$BC$36=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$36:$BC$36)))</f>
+        <v/>
+      </c>
+      <c r="N36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$36:$BC$36))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$36:$BC$36=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$36:$BC$36)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="I37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$37:$BC$37))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$37:$BC$37=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$37:$BC$37)))</f>
+        <v/>
+      </c>
+      <c r="J37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$37:$BC$37))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$37:$BC$37=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$37:$BC$37)))</f>
+        <v/>
+      </c>
+      <c r="K37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$37:$BC$37))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$37:$BC$37=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$37:$BC$37)))</f>
+        <v/>
+      </c>
+      <c r="L37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$37:$BC$37))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$37:$BC$37=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$37:$BC$37)))</f>
+        <v/>
+      </c>
+      <c r="M37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$37:$BC$37))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$37:$BC$37=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$37:$BC$37)))</f>
+        <v/>
+      </c>
+      <c r="N37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$37:$BC$37))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$37:$BC$37=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$37:$BC$37)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="I38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$38:$BC$38))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$38:$BC$38=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$38:$BC$38)))</f>
+        <v/>
+      </c>
+      <c r="J38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$38:$BC$38))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$38:$BC$38=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$38:$BC$38)))</f>
+        <v/>
+      </c>
+      <c r="K38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$38:$BC$38))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$38:$BC$38=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$38:$BC$38)))</f>
+        <v/>
+      </c>
+      <c r="L38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$38:$BC$38))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$38:$BC$38=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$38:$BC$38)))</f>
+        <v/>
+      </c>
+      <c r="M38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$38:$BC$38))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$38:$BC$38=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$38:$BC$38)))</f>
+        <v/>
+      </c>
+      <c r="N38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$38:$BC$38))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$38:$BC$38=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$38:$BC$38)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="I39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$39:$BC$39))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*(Marks!$B$39:$BC$39=1))/SUMPRODUCT((Marks!$B$2:$BC$2=I$3)*ISNUMBER(Marks!$B$39:$BC$39)))</f>
+        <v/>
+      </c>
+      <c r="J39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$39:$BC$39))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*(Marks!$B$39:$BC$39=1))/SUMPRODUCT((Marks!$B$2:$BC$2=J$3)*ISNUMBER(Marks!$B$39:$BC$39)))</f>
+        <v/>
+      </c>
+      <c r="K39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$39:$BC$39))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*(Marks!$B$39:$BC$39=1))/SUMPRODUCT((Marks!$B$2:$BC$2=K$3)*ISNUMBER(Marks!$B$39:$BC$39)))</f>
+        <v/>
+      </c>
+      <c r="L39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$39:$BC$39))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*(Marks!$B$39:$BC$39=1))/SUMPRODUCT((Marks!$B$2:$BC$2=L$3)*ISNUMBER(Marks!$B$39:$BC$39)))</f>
+        <v/>
+      </c>
+      <c r="M39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$39:$BC$39))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*(Marks!$B$39:$BC$39=1))/SUMPRODUCT((Marks!$B$2:$BC$2=M$3)*ISNUMBER(Marks!$B$39:$BC$39)))</f>
+        <v/>
+      </c>
+      <c r="N39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$39:$BC$39))=0,"",SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*(Marks!$B$39:$BC$39=1))/SUMPRODUCT((Marks!$B$2:$BC$2=N$3)*ISNUMBER(Marks!$B$39:$BC$39)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>The room</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Mean rating</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Right rate</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Rated 3 or 4, under half right</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Part 1. The week's rules, cold</t>
+        </is>
+      </c>
+      <c r="B43" s="7">
+        <f>IF(COUNT(B5:B39)=0,"",AVERAGE(B5:B39))</f>
+        <v/>
+      </c>
+      <c r="C43" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$14,MATCH(1,Tags!$A$5:$A$14,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D43">
+        <f>SUMPRODUCT((B5:B39&gt;=3)*ISNUMBER(I5:I39)*(I5:I39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Part 2. Where did the revenue go</t>
+        </is>
+      </c>
+      <c r="B44" s="7">
+        <f>IF(COUNT(C5:C39)=0,"",AVERAGE(C5:C39))</f>
+        <v/>
+      </c>
+      <c r="C44" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$14,MATCH(2,Tags!$A$5:$A$14,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D44">
+        <f>SUMPRODUCT((C5:C39&gt;=3)*ISNUMBER(J5:J39)*(J5:J39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Part 3. Rows you can trust</t>
+        </is>
+      </c>
+      <c r="B45" s="7">
+        <f>IF(COUNT(D5:D39)=0,"",AVERAGE(D5:D39))</f>
+        <v/>
+      </c>
+      <c r="C45" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$14,MATCH(3,Tags!$A$5:$A$14,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D45">
+        <f>SUMPRODUCT((D5:D39&gt;=3)*ISNUMBER(K5:K39)*(K5:K39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Part 4. Read the code, read the data</t>
+        </is>
+      </c>
+      <c r="B46" s="7">
+        <f>IF(COUNT(E5:E39)=0,"",AVERAGE(E5:E39))</f>
+        <v/>
+      </c>
+      <c r="C46" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$14,MATCH(4,Tags!$A$5:$A$14,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D46">
+        <f>SUMPRODUCT((E5:E39&gt;=3)*ISNUMBER(L5:L39)*(L5:L39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Part 5. Chance and a fair test</t>
+        </is>
+      </c>
+      <c r="B47" s="7">
+        <f>IF(COUNT(F5:F39)=0,"",AVERAGE(F5:F39))</f>
+        <v/>
+      </c>
+      <c r="C47" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$14,MATCH(5,Tags!$A$5:$A$14,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D47">
+        <f>SUMPRODUCT((F5:F39&gt;=3)*ISNUMBER(M5:M39)*(M5:M39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Part 6. The numbers</t>
+        </is>
+      </c>
+      <c r="B48" s="7">
+        <f>IF(COUNT(G5:G39)=0,"",AVERAGE(G5:G39))</f>
+        <v/>
+      </c>
+      <c r="C48" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$14,MATCH(6,Tags!$A$5:$A$14,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D48">
+        <f>SUMPRODUCT((G5:G39&gt;=3)*ISNUMBER(N5:N39)*(N5:N39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Saturday papers: relabel seven more-than-one items so no letter sits in every such key
Every more-than-one key in Week 1 held a and b, and every one in Week 2 held a, so ticking those
letters always scored. paper_edits.yaml gains an order edit, guarded by from_key, which relabels an
item's options and moves the key's letters and the reasons with them; four Week 1 items and three
Week 2 items use it, status proposed. distractor_audit.py now fails a recap paper where one letter
sits in every more-than-one key across four or more such items. Both provenance files record the
change, and exercise-builder states the rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7zaoR4dQ5pzBFnsX549JQ
</commit_message>
<xml_diff>
--- a/content/W01/SAT/answer-key/C2_W01_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W01/SAT/answer-key/C2_W01_SAT_item_analysis_TRAINER.xlsx
@@ -4762,7 +4762,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>a, b, c</t>
+          <t>b, c, d</t>
         </is>
       </c>
       <c r="G20">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>a, b, c</t>
+          <t>a, c, d</t>
         </is>
       </c>
       <c r="G30">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>a, b, c</t>
+          <t>b, c, d</t>
         </is>
       </c>
       <c r="G48">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>a, b, d</t>
+          <t>a, c, d</t>
         </is>
       </c>
       <c r="G49">

</xml_diff>

<commit_message>
W01 SAT: each part named by the question it asks, and each opening says who needs the answer
Part titles become plain questions (where Kalpa's revenue went between the
quarters; whether Kalpa booked Rs 2.1 or 1.9 crore in the first quarter;
whether the Retail-Plus fall is more than chance and what Meera's note says;
which check would have caught the misleading number in five public cases;
whether a delivery company's offer raised spending and its agent's numbers are
right). The openings name who needs each answer and what rides on it, define
booked value as the dossier's GMV, the quarters, the ladder and profiling, and
Kavya's test becomes flips of each member's own two quarters. Paper, key, Word
files and workbook rebuilt with the builder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K8RZ1KXh1k8mKVCEBq4phk
</commit_message>
<xml_diff>
--- a/content/W01/SAT/answer-key/C2_W01_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W01/SAT/answer-key/C2_W01_SAT_item_analysis_TRAINER.xlsx
@@ -6095,7 +6095,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Part 1. Where the revenue went</t>
+          <t>Part 1. Where did Kalpa's revenue go between the first quarter and the second?</t>
         </is>
       </c>
       <c r="C9">
@@ -6113,7 +6113,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Part 2. Which Q1 figure is right</t>
+          <t>Part 2. Did Kalpa book Rs 2.1 crore in the first quarter, or Rs 1.9 crore?</t>
         </is>
       </c>
       <c r="C10">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Part 3. Real, or the wobble</t>
+          <t>Part 3. Is the Retail-Plus fall more than chance, and what should Meera's note say?</t>
         </is>
       </c>
       <c r="C11">
@@ -6149,7 +6149,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Part 4. The same traps, in public</t>
+          <t>Part 4. Which check would have caught the misleading number in five public cases?</t>
         </is>
       </c>
       <c r="C12">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Part 5. An offer, an agent and its logs</t>
+          <t>Part 5. Did a delivery company's offer raise spending, and are its AI agent's numbers right?</t>
         </is>
       </c>
       <c r="C13">
@@ -8164,7 +8164,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Part 1. Where the revenue went</t>
+          <t>Part 1. Where did Kalpa's revenue go between the first quarter and the second?</t>
         </is>
       </c>
       <c r="B43" s="7">
@@ -8183,7 +8183,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Part 2. Which Q1 figure is right</t>
+          <t>Part 2. Did Kalpa book Rs 2.1 crore in the first quarter, or Rs 1.9 crore?</t>
         </is>
       </c>
       <c r="B44" s="7">
@@ -8202,7 +8202,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Part 3. Real, or the wobble</t>
+          <t>Part 3. Is the Retail-Plus fall more than chance, and what should Meera's note say?</t>
         </is>
       </c>
       <c r="B45" s="7">
@@ -8221,7 +8221,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Part 4. The same traps, in public</t>
+          <t>Part 4. Which check would have caught the misleading number in five public cases?</t>
         </is>
       </c>
       <c r="B46" s="7">
@@ -8240,7 +8240,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Part 5. An offer, an agent and its logs</t>
+          <t>Part 5. Did a delivery company's offer raise spending, and are its AI agent's numbers right?</t>
         </is>
       </c>
       <c r="B47" s="7">

</xml_diff>